<commit_message>
Added log download page
</commit_message>
<xml_diff>
--- a/src/static/contact_list.xlsx
+++ b/src/static/contact_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Myat\Avatar\standard_aiserver\src\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEAB4FA3-51E7-415D-ACAD-E627D1731205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA74F9A-9325-4950-B84F-12E7E7FEB37C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Branch Name</t>
     <phoneticPr fontId="1"/>
@@ -56,10 +56,6 @@
     <rPh sb="2" eb="4">
       <t>シテン</t>
     </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>鳥羽　光生</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -396,7 +392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="22.1640625" customWidth="1"/>
@@ -420,7 +416,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>7075232221</v>
@@ -428,23 +424,12 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3">
-        <v>7075232221</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4">
         <v>7075232221</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add changes for Hokkaido Glory
</commit_message>
<xml_diff>
--- a/src/static/contact_list.xlsx
+++ b/src/static/contact_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Myat\Avatar\standard_aiserver\src\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEAB4FA3-51E7-415D-ACAD-E627D1731205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381D785E-E479-4BDD-AB30-327E30B40B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Branch Name</t>
     <phoneticPr fontId="1"/>
@@ -39,36 +39,19 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>東京本社</t>
-    <rPh sb="0" eb="2">
-      <t>トウキョウ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ホンシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>札幌支店</t>
-    <rPh sb="0" eb="2">
-      <t>サッポロ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>シテン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>鳥羽　光生</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>土橋 旭</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>川頭  美和</t>
-    <phoneticPr fontId="1"/>
+    <t>札幌本社</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>阿部部⾧</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>旭川支店</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>須藤支店⾧</t>
   </si>
 </sst>
 </file>
@@ -396,7 +379,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="22.1640625" customWidth="1"/>
@@ -420,32 +403,21 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>7075232221</v>
+        <v>12345678</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
       <c r="C3">
-        <v>7075232221</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4">
-        <v>7075232221</v>
+        <v>12345678</v>
       </c>
     </row>
   </sheetData>

</xml_diff>